<commit_message>
Change Button_excecl_all to Button clear
</commit_message>
<xml_diff>
--- a/excel_payment.xlsx
+++ b/excel_payment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20386"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20388"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jackey\Desktop\github\work-order\app\dist\main\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jackey\Desktop\github\work-order\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBEEE61B-8B44-4017-BE05-03A93134ACBE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3177E884-5B65-41FC-B465-33C7D71D0C12}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView showHorizontalScroll="0" showSheetTabs="0" xWindow="32767" yWindow="32767" windowWidth="24180" windowHeight="13053" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -86,29 +86,31 @@
     <t>計價</t>
   </si>
   <si>
-    <t>特殊計價</t>
+    <t>製作金額</t>
+  </si>
+  <si>
+    <t>稅額</t>
+  </si>
+  <si>
+    <t>製作總價</t>
+  </si>
+  <si>
+    <t>匯款資料:
+銀行:合作金庫-永吉分行(銀行代號006)
+帳號:0969-717-059213             戶名:彩意企業有限公司</t>
+  </si>
+  <si>
+    <t>公司統編:</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">本報價單務必請承辦人員確認製作與製作金額後簽章並回本公司。
 本報價單請款方式為:於交貨日起算開立30日之內付款，務請貴公司配合請款條件，謝謝。
 </t>
-  </si>
-  <si>
-    <t>製作金額</t>
-  </si>
-  <si>
-    <t>稅額</t>
-  </si>
-  <si>
-    <t>製作總價</t>
-  </si>
-  <si>
-    <t>匯款資料:
-銀行:合作金庫-永吉分行(銀行代號006)
-帳號:0969-717-059213             戶名:彩意企業有限公司</t>
-  </si>
-  <si>
-    <t>公司統編:</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>備料計價</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -520,16 +522,21 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
@@ -537,43 +544,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -877,44 +879,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="33.700000000000003" customHeight="1" thickBot="1">
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
       <c r="E1" s="17"/>
-      <c r="F1" s="41" t="s">
+      <c r="F1" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="49" t="s">
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="40"/>
+      <c r="L1" s="29"/>
     </row>
     <row r="2" spans="1:13" ht="17" customHeight="1">
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
       <c r="E2" s="20"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="40"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
     </row>
     <row r="3" spans="1:13" ht="32.700000000000003" customHeight="1">
       <c r="B3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="51"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="53"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="46"/>
       <c r="F3" s="27" t="s">
         <v>4</v>
       </c>
@@ -935,11 +937,11 @@
       <c r="B4" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="51"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="53"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="46"/>
       <c r="H4" s="23" t="s">
         <v>8</v>
       </c>
@@ -948,36 +950,36 @@
         <v>9</v>
       </c>
       <c r="K4" s="22"/>
-      <c r="L4" s="46"/>
-      <c r="M4" s="45"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="28"/>
     </row>
     <row r="5" spans="1:13" ht="33" customHeight="1">
       <c r="B5" s="21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C5" s="22"/>
-      <c r="D5" s="43" t="s">
+      <c r="D5" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="43"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="44"/>
-      <c r="J5" s="44"/>
-      <c r="K5" s="44"/>
-      <c r="L5" s="33"/>
-      <c r="M5" s="40"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
+      <c r="H5" s="53"/>
+      <c r="I5" s="53"/>
+      <c r="J5" s="53"/>
+      <c r="K5" s="53"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="29"/>
     </row>
     <row r="6" spans="1:13" ht="30" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="47" t="s">
+      <c r="C6" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="48"/>
+      <c r="D6" s="33"/>
       <c r="E6" s="13" t="s">
         <v>14</v>
       </c>
@@ -1000,14 +1002,14 @@
         <v>19</v>
       </c>
       <c r="L6" s="25" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="26"/>
-      <c r="C7" s="42"/>
-      <c r="D7" s="42"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
       <c r="E7" s="26"/>
       <c r="F7" s="26"/>
       <c r="G7" s="26"/>
@@ -1020,8 +1022,8 @@
     <row r="8" spans="1:13" ht="30" customHeight="1">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
       <c r="E8" s="26"/>
       <c r="F8" s="26"/>
       <c r="G8" s="26"/>
@@ -1034,8 +1036,8 @@
     <row r="9" spans="1:13" ht="30" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="26"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
       <c r="E9" s="26"/>
       <c r="F9" s="26"/>
       <c r="G9" s="26"/>
@@ -1048,8 +1050,8 @@
     <row r="10" spans="1:13" ht="30" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="26"/>
-      <c r="C10" s="42"/>
-      <c r="D10" s="42"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
       <c r="E10" s="26"/>
       <c r="F10" s="26"/>
       <c r="G10" s="26"/>
@@ -1062,8 +1064,8 @@
     <row r="11" spans="1:13" ht="30" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="26"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
       <c r="E11" s="26"/>
       <c r="F11" s="26"/>
       <c r="G11" s="26"/>
@@ -1076,8 +1078,8 @@
     <row r="12" spans="1:13" ht="30" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="26"/>
-      <c r="C12" s="42"/>
-      <c r="D12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
       <c r="E12" s="26"/>
       <c r="F12" s="26"/>
       <c r="G12" s="26"/>
@@ -1090,8 +1092,8 @@
     <row r="13" spans="1:13" ht="30" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="26"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
       <c r="E13" s="26"/>
       <c r="F13" s="26"/>
       <c r="G13" s="26"/>
@@ -1104,8 +1106,8 @@
     <row r="14" spans="1:13" ht="30" customHeight="1">
       <c r="A14" s="1"/>
       <c r="B14" s="26"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
       <c r="E14" s="26"/>
       <c r="F14" s="26"/>
       <c r="G14" s="26"/>
@@ -1117,8 +1119,8 @@
     </row>
     <row r="15" spans="1:13" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B15" s="26"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
       <c r="E15" s="26"/>
       <c r="F15" s="26"/>
       <c r="G15" s="26"/>
@@ -1130,8 +1132,8 @@
     </row>
     <row r="16" spans="1:13" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B16" s="26"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
       <c r="E16" s="26"/>
       <c r="F16" s="26"/>
       <c r="G16" s="26"/>
@@ -1144,8 +1146,8 @@
     <row r="17" spans="1:12" ht="30" customHeight="1">
       <c r="A17" s="1"/>
       <c r="B17" s="26"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
       <c r="E17" s="26"/>
       <c r="F17" s="26"/>
       <c r="G17" s="26"/>
@@ -1157,8 +1159,8 @@
     </row>
     <row r="18" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B18" s="26"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
       <c r="E18" s="26"/>
       <c r="F18" s="26"/>
       <c r="G18" s="26"/>
@@ -1170,8 +1172,8 @@
     </row>
     <row r="19" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B19" s="26"/>
-      <c r="C19" s="42"/>
-      <c r="D19" s="42"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
       <c r="E19" s="26"/>
       <c r="F19" s="26"/>
       <c r="G19" s="26"/>
@@ -1183,8 +1185,8 @@
     </row>
     <row r="20" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B20" s="26"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
       <c r="E20" s="26"/>
       <c r="F20" s="26"/>
       <c r="G20" s="26"/>
@@ -1196,8 +1198,8 @@
     </row>
     <row r="21" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B21" s="26"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
       <c r="E21" s="26"/>
       <c r="F21" s="26"/>
       <c r="G21" s="26"/>
@@ -1208,118 +1210,118 @@
       <c r="L21" s="26"/>
     </row>
     <row r="22" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="B22" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="30"/>
+      <c r="B22" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="40"/>
       <c r="G22" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="L22" s="6"/>
     </row>
     <row r="23" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="B23" s="31"/>
-      <c r="C23" s="32"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32"/>
-      <c r="F23" s="33"/>
+      <c r="B23" s="41"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="31"/>
       <c r="G23" s="7"/>
-      <c r="H23" s="50"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
-      <c r="K23" s="35"/>
-      <c r="L23" s="36"/>
+      <c r="H23" s="35"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
+      <c r="K23" s="36"/>
+      <c r="L23" s="37"/>
     </row>
     <row r="24" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B24" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="38"/>
-      <c r="J24" s="38"/>
-      <c r="K24" s="38"/>
-      <c r="L24" s="30"/>
+      <c r="B24" s="49" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="38"/>
+      <c r="I24" s="39"/>
+      <c r="J24" s="39"/>
+      <c r="K24" s="39"/>
+      <c r="L24" s="40"/>
     </row>
     <row r="25" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B25" s="37"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="37"/>
-      <c r="I25" s="38"/>
-      <c r="J25" s="38"/>
-      <c r="K25" s="38"/>
-      <c r="L25" s="30"/>
+      <c r="B25" s="38"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="39"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="39"/>
+      <c r="J25" s="39"/>
+      <c r="K25" s="39"/>
+      <c r="L25" s="40"/>
     </row>
     <row r="26" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B26" s="37"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="37"/>
-      <c r="I26" s="38"/>
-      <c r="J26" s="38"/>
-      <c r="K26" s="38"/>
-      <c r="L26" s="30"/>
+      <c r="B26" s="38"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="38"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="39"/>
+      <c r="K26" s="39"/>
+      <c r="L26" s="40"/>
     </row>
     <row r="27" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B27" s="37"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="37"/>
-      <c r="I27" s="38"/>
-      <c r="J27" s="38"/>
-      <c r="K27" s="38"/>
-      <c r="L27" s="30"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="39"/>
+      <c r="K27" s="39"/>
+      <c r="L27" s="40"/>
     </row>
     <row r="28" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B28" s="37"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="37"/>
-      <c r="I28" s="38"/>
-      <c r="J28" s="38"/>
-      <c r="K28" s="38"/>
-      <c r="L28" s="30"/>
+      <c r="B28" s="38"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="39"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="39"/>
+      <c r="K28" s="39"/>
+      <c r="L28" s="40"/>
     </row>
     <row r="29" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B29" s="31"/>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="31"/>
-      <c r="I29" s="32"/>
-      <c r="J29" s="32"/>
-      <c r="K29" s="32"/>
-      <c r="L29" s="33"/>
+      <c r="B29" s="41"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="42"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="41"/>
+      <c r="I29" s="42"/>
+      <c r="J29" s="42"/>
+      <c r="K29" s="42"/>
+      <c r="L29" s="31"/>
     </row>
     <row r="30" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
       <c r="B30" s="8"/>
@@ -1355,6 +1357,18 @@
     <row r="38"/>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="B22:F23"/>
+    <mergeCell ref="B24:G29"/>
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="F1:J2"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:K5"/>
     <mergeCell ref="M4:M5"/>
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="C6:D6"/>
@@ -1371,18 +1385,6 @@
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="C3:E3"/>
-    <mergeCell ref="B22:F23"/>
-    <mergeCell ref="B24:G29"/>
-    <mergeCell ref="B1:D2"/>
-    <mergeCell ref="F1:J2"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:K5"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Update payment Excel template
</commit_message>
<xml_diff>
--- a/excel_payment.xlsx
+++ b/excel_payment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20390"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jackey\Desktop\github\work-order\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACA69195-7BB4-46D7-A806-AD102AA0DCAF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C17C7EED-336D-4550-9BC7-FCBF119F9221}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView showHorizontalScroll="0" showSheetTabs="0" xWindow="32767" yWindow="32767" windowWidth="24180" windowHeight="13053" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -92,11 +92,6 @@
     <t>製作總價</t>
   </si>
   <si>
-    <t>匯款資料:
-銀行:合作金庫-永吉分行(銀行代號006)
-帳號:0969-717-059213             戶名:彩意企業有限公司</t>
-  </si>
-  <si>
     <t>公司統編:</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -112,6 +107,12 @@
   </si>
   <si>
     <t>報價單</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>匯款資料:
+銀行:合作金庫-松山分行(銀行代號006)
+帳號:0969-717-059213             戶名:彩意企業有限公司</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -534,12 +535,43 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -560,9 +592,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -570,34 +599,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -901,44 +902,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="33.700000000000003" customHeight="1" thickBot="1">
-      <c r="B1" s="58" t="s">
+      <c r="B1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
       <c r="E1" s="17"/>
-      <c r="F1" s="59" t="s">
+      <c r="F1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="34" t="s">
-        <v>26</v>
-      </c>
-      <c r="L1" s="29"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="49" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="40"/>
     </row>
     <row r="2" spans="1:13" ht="17" customHeight="1">
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
       <c r="E2" s="20"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40"/>
     </row>
     <row r="3" spans="1:13" ht="32.700000000000003" customHeight="1">
       <c r="B3" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="45"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="61"/>
       <c r="F3" s="27" t="s">
         <v>3</v>
       </c>
@@ -959,11 +960,11 @@
       <c r="B4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="47"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="61"/>
       <c r="H4" s="23" t="s">
         <v>7</v>
       </c>
@@ -972,36 +973,36 @@
         <v>8</v>
       </c>
       <c r="K4" s="22"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="28"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="45"/>
     </row>
     <row r="5" spans="1:13" ht="33" customHeight="1">
       <c r="B5" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="22"/>
-      <c r="D5" s="60" t="s">
+      <c r="D5" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="60"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="61"/>
-      <c r="H5" s="61"/>
-      <c r="I5" s="61"/>
-      <c r="J5" s="61"/>
-      <c r="K5" s="61"/>
-      <c r="L5" s="31"/>
-      <c r="M5" s="29"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="40"/>
     </row>
     <row r="6" spans="1:13" ht="30" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="33"/>
+      <c r="D6" s="48"/>
       <c r="E6" s="13" t="s">
         <v>13</v>
       </c>
@@ -1024,14 +1025,14 @@
         <v>18</v>
       </c>
       <c r="L6" s="25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="26"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
       <c r="E7" s="26"/>
       <c r="F7" s="26"/>
       <c r="G7" s="26"/>
@@ -1044,8 +1045,8 @@
     <row r="8" spans="1:13" ht="30" customHeight="1">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
       <c r="E8" s="26"/>
       <c r="F8" s="26"/>
       <c r="G8" s="26"/>
@@ -1058,8 +1059,8 @@
     <row r="9" spans="1:13" ht="30" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="26"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
       <c r="E9" s="26"/>
       <c r="F9" s="26"/>
       <c r="G9" s="26"/>
@@ -1072,8 +1073,8 @@
     <row r="10" spans="1:13" ht="30" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="26"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
       <c r="E10" s="26"/>
       <c r="F10" s="26"/>
       <c r="G10" s="26"/>
@@ -1086,8 +1087,8 @@
     <row r="11" spans="1:13" ht="30" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="26"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
       <c r="E11" s="26"/>
       <c r="F11" s="26"/>
       <c r="G11" s="26"/>
@@ -1100,8 +1101,8 @@
     <row r="12" spans="1:13" ht="30" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="26"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
       <c r="E12" s="26"/>
       <c r="F12" s="26"/>
       <c r="G12" s="26"/>
@@ -1114,8 +1115,8 @@
     <row r="13" spans="1:13" ht="30" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="26"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
       <c r="E13" s="26"/>
       <c r="F13" s="26"/>
       <c r="G13" s="26"/>
@@ -1128,8 +1129,8 @@
     <row r="14" spans="1:13" ht="30" customHeight="1">
       <c r="A14" s="1"/>
       <c r="B14" s="26"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
       <c r="E14" s="26"/>
       <c r="F14" s="26"/>
       <c r="G14" s="26"/>
@@ -1141,8 +1142,8 @@
     </row>
     <row r="15" spans="1:13" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B15" s="26"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="44"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
       <c r="E15" s="26"/>
       <c r="F15" s="26"/>
       <c r="G15" s="26"/>
@@ -1154,8 +1155,8 @@
     </row>
     <row r="16" spans="1:13" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B16" s="26"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="44"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
       <c r="E16" s="26"/>
       <c r="F16" s="26"/>
       <c r="G16" s="26"/>
@@ -1168,8 +1169,8 @@
     <row r="17" spans="1:12" ht="30" customHeight="1">
       <c r="A17" s="1"/>
       <c r="B17" s="26"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
       <c r="E17" s="26"/>
       <c r="F17" s="26"/>
       <c r="G17" s="26"/>
@@ -1181,8 +1182,8 @@
     </row>
     <row r="18" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B18" s="26"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="44"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
       <c r="E18" s="26"/>
       <c r="F18" s="26"/>
       <c r="G18" s="26"/>
@@ -1194,8 +1195,8 @@
     </row>
     <row r="19" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B19" s="26"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
       <c r="E19" s="26"/>
       <c r="F19" s="26"/>
       <c r="G19" s="26"/>
@@ -1207,8 +1208,8 @@
     </row>
     <row r="20" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B20" s="26"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
       <c r="E20" s="26"/>
       <c r="F20" s="26"/>
       <c r="G20" s="26"/>
@@ -1220,8 +1221,8 @@
     </row>
     <row r="21" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="B21" s="26"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
       <c r="E21" s="26"/>
       <c r="F21" s="26"/>
       <c r="G21" s="26"/>
@@ -1232,13 +1233,13 @@
       <c r="L21" s="26"/>
     </row>
     <row r="22" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="B22" s="48" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" s="49"/>
-      <c r="D22" s="49"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="50"/>
+      <c r="B22" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="30"/>
       <c r="G22" s="10" t="s">
         <v>19</v>
       </c>
@@ -1253,97 +1254,97 @@
       <c r="L22" s="6"/>
     </row>
     <row r="23" spans="1:12" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="B23" s="51"/>
-      <c r="C23" s="52"/>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="31"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="33"/>
       <c r="G23" s="7"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="36"/>
-      <c r="J23" s="36"/>
-      <c r="K23" s="36"/>
-      <c r="L23" s="37"/>
+      <c r="H23" s="50"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="51"/>
+      <c r="K23" s="51"/>
+      <c r="L23" s="52"/>
     </row>
     <row r="24" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B24" s="53" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="54"/>
-      <c r="D24" s="54"/>
-      <c r="E24" s="54"/>
-      <c r="F24" s="54"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="39"/>
-      <c r="J24" s="39"/>
-      <c r="K24" s="39"/>
-      <c r="L24" s="40"/>
+      <c r="B24" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="54"/>
+      <c r="J24" s="54"/>
+      <c r="K24" s="54"/>
+      <c r="L24" s="55"/>
     </row>
     <row r="25" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B25" s="56"/>
-      <c r="C25" s="57"/>
-      <c r="D25" s="57"/>
-      <c r="E25" s="57"/>
-      <c r="F25" s="57"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="39"/>
-      <c r="J25" s="39"/>
-      <c r="K25" s="39"/>
-      <c r="L25" s="40"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="53"/>
+      <c r="I25" s="54"/>
+      <c r="J25" s="54"/>
+      <c r="K25" s="54"/>
+      <c r="L25" s="55"/>
     </row>
     <row r="26" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B26" s="56"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="50"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="39"/>
-      <c r="J26" s="39"/>
-      <c r="K26" s="39"/>
-      <c r="L26" s="40"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="54"/>
+      <c r="J26" s="54"/>
+      <c r="K26" s="54"/>
+      <c r="L26" s="55"/>
     </row>
     <row r="27" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B27" s="56"/>
-      <c r="C27" s="57"/>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="57"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="38"/>
-      <c r="I27" s="39"/>
-      <c r="J27" s="39"/>
-      <c r="K27" s="39"/>
-      <c r="L27" s="40"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="53"/>
+      <c r="I27" s="54"/>
+      <c r="J27" s="54"/>
+      <c r="K27" s="54"/>
+      <c r="L27" s="55"/>
     </row>
     <row r="28" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B28" s="56"/>
-      <c r="C28" s="57"/>
-      <c r="D28" s="57"/>
-      <c r="E28" s="57"/>
-      <c r="F28" s="57"/>
-      <c r="G28" s="50"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="39"/>
-      <c r="J28" s="39"/>
-      <c r="K28" s="39"/>
-      <c r="L28" s="40"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="53"/>
+      <c r="I28" s="54"/>
+      <c r="J28" s="54"/>
+      <c r="K28" s="54"/>
+      <c r="L28" s="55"/>
     </row>
     <row r="29" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
-      <c r="B29" s="51"/>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
-      <c r="E29" s="52"/>
-      <c r="F29" s="52"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="41"/>
-      <c r="I29" s="42"/>
-      <c r="J29" s="42"/>
-      <c r="K29" s="42"/>
-      <c r="L29" s="43"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="57"/>
+      <c r="J29" s="57"/>
+      <c r="K29" s="57"/>
+      <c r="L29" s="58"/>
     </row>
     <row r="30" spans="1:12" s="1" customFormat="1" ht="12.7" customHeight="1">
       <c r="B30" s="8"/>
@@ -1379,18 +1380,6 @@
     <row r="38"/>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="B22:F23"/>
-    <mergeCell ref="B24:G29"/>
-    <mergeCell ref="B1:D2"/>
-    <mergeCell ref="F1:J2"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:K5"/>
     <mergeCell ref="M4:M5"/>
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="C6:D6"/>
@@ -1407,6 +1396,18 @@
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="C3:E3"/>
+    <mergeCell ref="B22:F23"/>
+    <mergeCell ref="B24:G29"/>
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="F1:J2"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:K5"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>